<commit_message>
fixed small changes in the timetable unscheduled classes since it wasn't showing the uncheduled TP , next step is to fix groups of type specialite and make them appear on the timetable
</commit_message>
<xml_diff>
--- a/modele/Tous_les_Emplois_du_Temps.xlsx
+++ b/modele/Tous_les_Emplois_du_Temps.xlsx
@@ -88,14 +88,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
-        <bgColor rgb="00FFE699"/>
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
-        <bgColor rgb="00C6E0B4"/>
+        <fgColor rgb="00FFE699"/>
+        <bgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,10 +137,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -582,7 +582,49 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD2
+Prof: Esseyssah
+Salle: 102</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD1
+Prof: Kaber
+Salle: 102 /// [SYR211] Systèmes d’exploitation
+(TP) - TD2
+Prof: Debagh
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
@@ -590,35 +632,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(TP) - TD1
-Prof: Sidi Mouhamed
-Salle: 102 /// [DEV210] Programmation Python
-(TP) - TD2
-Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>[SPEC211] PI 1
 (CM)
@@ -626,8 +640,115 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD1
@@ -638,28 +759,24 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
 Salle: 101</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -667,63 +784,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Debagh
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>[DPR212] Projet Personnel et Professionnel II
 (CM)
@@ -731,64 +792,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD1
-Prof: Kaber
-Salle: 102 /// [SYR211] Systèmes d’exploitation
-(TP) - TD2
-Prof: Debagh
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -876,13 +880,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -894,13 +898,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -912,13 +916,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -930,13 +934,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -948,13 +952,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1042,13 +1046,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1060,13 +1064,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1078,13 +1082,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1096,13 +1100,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1114,13 +1118,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1208,13 +1212,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1226,13 +1230,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1244,13 +1248,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1262,13 +1266,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1280,13 +1284,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1374,13 +1378,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1392,13 +1396,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1410,13 +1414,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1428,13 +1432,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1446,13 +1450,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1540,13 +1544,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1558,13 +1562,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1576,13 +1580,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1594,13 +1598,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1612,13 +1616,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1706,13 +1710,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1724,13 +1728,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1742,13 +1746,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1760,13 +1764,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1778,13 +1782,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1872,13 +1876,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1890,13 +1894,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1908,13 +1912,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1926,13 +1930,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1944,13 +1948,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2038,13 +2042,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2056,13 +2060,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2074,13 +2078,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2092,13 +2096,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2110,13 +2114,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2204,13 +2208,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2222,13 +2226,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2240,13 +2244,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2258,13 +2262,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2276,13 +2280,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2370,13 +2374,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2388,13 +2392,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2406,13 +2410,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2424,13 +2428,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2442,13 +2446,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2536,15 +2540,16 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>[MAI211] Probabilités et Statistiques
 (CM)
@@ -2552,8 +2557,150 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr"/>
       <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Sidi Soueina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD4
+Prof: Esseyssah
+Salle: 102</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(TP) - TD3
+Prof: Debagh
+Salle: 102 /// [DEV211] Langages Web
+(TP) - TD4
+Prof: Aicha
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD3
@@ -2564,8 +2711,19 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
@@ -2573,35 +2731,15 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
 Salle: 201</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -2609,75 +2747,9 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(TP) - TD3
-Prof: Debagh
-Salle: 102 /// [DEV210] Programmation Python
-(TP) - TD4
-Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Sidi Soueina
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -2685,54 +2757,7 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(TP) - TD4
-Prof: Aicha
-Salle: 102</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2820,13 +2845,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2838,13 +2863,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2856,13 +2881,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2874,13 +2899,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2892,13 +2917,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2986,13 +3011,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3004,13 +3029,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3022,13 +3047,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3040,13 +3065,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3058,13 +3083,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3152,13 +3177,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3170,13 +3195,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3188,13 +3213,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3206,13 +3231,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3224,13 +3249,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3318,13 +3343,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3336,13 +3361,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3354,13 +3379,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3372,13 +3397,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3390,20 +3415,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online)
-Prof: Med Lemine
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3491,13 +3509,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3509,13 +3527,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3527,13 +3545,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3545,13 +3563,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3563,13 +3581,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3657,135 +3675,15 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Moussa
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD5
-Prof: Kaber
-Salle: 104 /// [SYR211] Systèmes d’exploitation
-(TP) - TD6
-Prof: Debagh
-Salle: 204</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Marba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Cheiba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
 Salle: 201</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD5
@@ -3796,67 +3694,198 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Cheiba
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Marba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Meya
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 201</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
 (TP) - TD5
-Prof: Moussa
-Salle: 102 /// [DEV210] Programmation Python
+Prof: Kaber
+Salle: 104 /// [DEV210] Programmation Python
 (TP) - TD6
 Prof: Mahfoudh
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
+Salle: 204</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
 Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
 Salle: 201</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3944,15 +3973,156 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
 Prof: Habeb
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD8
+Prof: Mahfoudh
+Salle: 104</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD7
+Prof: Kaber
+Salle: 103 /// [SYR211] Systèmes d’exploitation
+(TP) - TD8
+Prof: Debagh
+Salle: 104</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
 Salle: 203</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(TD)
+Prof: Marba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Cheiba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD7
@@ -3963,145 +4133,25 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Moussa
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(TP) - TD7
-Prof: Moussa
-Salle: 102 /// [DEV210] Programmation Python
-(TP) - TD8
-Prof: Mahfoudh
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Cheiba
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4115,33 +4165,21 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD7
-Prof: Kaber
-Salle: 103 /// [SYR211] Systèmes d’exploitation
-(TP) - TD8
-Prof: Debagh
-Salle: 104</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
           <t>[SPEC211] PI 1
 (CM)
 Prof: Encadreur
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(TD)
-Prof: Marba
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr">
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Meya
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM Online)
@@ -4149,8 +4187,17 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4238,13 +4285,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4256,13 +4303,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4274,13 +4321,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4292,13 +4339,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4310,13 +4357,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4404,13 +4451,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4422,13 +4469,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4440,13 +4487,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4458,13 +4505,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4476,13 +4523,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4570,13 +4617,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4588,13 +4635,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4606,13 +4653,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4624,13 +4671,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4642,13 +4689,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4736,13 +4783,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4754,13 +4801,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4772,13 +4819,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4790,13 +4837,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4808,13 +4855,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4902,13 +4949,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4920,13 +4967,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4938,13 +4985,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4956,13 +5003,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4974,13 +5021,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>

</xml_diff>

<commit_message>
Fixed the groups of type specialite but still haven't test it yet so will continue in another time for now will take it as it completed
</commit_message>
<xml_diff>
--- a/modele/Tous_les_Emplois_du_Temps.xlsx
+++ b/modele/Tous_les_Emplois_du_Temps.xlsx
@@ -88,14 +88,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
-        <bgColor rgb="00C6E0B4"/>
+        <fgColor rgb="00FFE699"/>
+        <bgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
-        <bgColor rgb="00FFE699"/>
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,13 +137,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -582,8 +582,22 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
+Salle: 101</t>
+        </is>
+      </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
@@ -592,7 +606,150 @@
 Salle: 102</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI2
+Prof: Med Lemine
+Salle: 201 /// [RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Sidi Soueina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD1
@@ -603,140 +760,7 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Debagh
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -759,24 +783,27 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Hassina
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI1
+Prof: Med Lemine
+Salle: 101 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
 Salle: 101</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -784,15 +811,8 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Sidi Soueina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -880,13 +900,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -898,13 +918,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -916,13 +936,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -934,13 +954,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -952,13 +972,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1046,13 +1066,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1064,13 +1084,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1082,13 +1102,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1100,13 +1120,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1118,13 +1138,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1212,13 +1232,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1230,13 +1250,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1248,13 +1268,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1266,13 +1286,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1284,13 +1304,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1378,13 +1398,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1396,13 +1416,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1414,13 +1434,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1432,13 +1452,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1450,13 +1470,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1544,13 +1564,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1562,13 +1582,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1580,13 +1600,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1598,13 +1618,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1616,13 +1636,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1710,13 +1730,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1728,13 +1748,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1746,13 +1766,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1764,13 +1784,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1782,13 +1802,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1876,13 +1896,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1894,13 +1914,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1912,13 +1932,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1930,13 +1950,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1948,13 +1968,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2042,13 +2062,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2060,13 +2080,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2078,13 +2098,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2096,13 +2116,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2114,13 +2134,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2208,13 +2228,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2226,13 +2246,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2244,13 +2264,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2262,13 +2282,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2280,13 +2300,20 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM)
+Prof: Med Lemine
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2374,13 +2401,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2392,13 +2419,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2410,13 +2437,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2428,13 +2455,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2446,13 +2473,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2540,41 +2567,44 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
 Prof: Tah
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
 Salle: 101</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD3
+Prof: Kaber
+Salle: 102 /// [SYR211] Systèmes d’exploitation
+(TP) - TD4
+Prof: Debagh
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>[DPR212] Projet Personnel et Professionnel II
 (CM)
 Prof: Sidi Soueina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2586,28 +2616,27 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI2
+Prof: Med Lemine
+Salle: 201 /// [RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101 /// [DEV210] Programmation Python
 (TP) - TD4
 Prof: Esseyssah
 Salle: 102</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
 Salle: 201</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -2621,16 +2650,16 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Debagh
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
 Salle: 201</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2642,7 +2671,7 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -2650,16 +2679,118 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>[MAI212] Préparation à la certification PIX 2
 (CM)
 Prof: Hassina
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
 Salle: 101</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI1
+Prof: Med Lemine
+Salle: 101 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
@@ -2667,97 +2798,9 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD3
-Prof: Kaber
-Salle: 102 /// [SYR211] Systèmes d’exploitation
-(TP) - TD4
-Prof: Debagh
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2845,13 +2888,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2863,13 +2906,20 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(CM)
+Prof: Souvi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2881,13 +2931,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2899,13 +2949,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2917,13 +2967,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3011,13 +3061,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3029,13 +3079,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3047,13 +3097,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3065,13 +3115,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3083,13 +3133,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3177,13 +3227,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3195,13 +3245,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3213,13 +3263,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3231,13 +3281,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3249,13 +3299,20 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>[CNM210] CMS et PAO
+(CM)
+Prof: Cheikhani
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3343,13 +3400,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3361,13 +3418,20 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM)
+Prof: Med Lemine
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3379,13 +3443,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3397,13 +3461,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3415,13 +3479,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3509,13 +3573,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3527,13 +3591,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3545,13 +3609,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3563,13 +3627,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3581,13 +3645,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3675,12 +3739,12 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Moussa
-Salle: 201</t>
+Salle: 202</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -3694,16 +3758,57 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
 Salle: 201</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI2
+Prof: Med Lemine
+Salle: 201 /// [RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>[MAI211] Probabilités et Statistiques
 (CM)
@@ -3711,20 +3816,28 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Meya
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -3732,15 +3845,62 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM)
 Prof: Marba
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
 Salle: 202</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -3748,109 +3908,9 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Meya
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3873,19 +3933,43 @@
 Salle: 204</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI1
+Prof: Med Lemine
+Salle: 101 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
 Salle: 201</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3973,20 +4057,20 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
 Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(TP) - TD8
-Prof: Mahfoudh
-Salle: 104</t>
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(TD)
+Prof: Marba
+Salle: 201</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -4000,31 +4084,31 @@
 Salle: 104</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
 Salle: 202</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Moussa
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4036,34 +4120,44 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI2
+Prof: Med Lemine
+Salle: 201 /// [RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
 Prof: Hatabi
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
 Salle: 203</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(TD)
-Prof: Marba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4075,16 +4169,9 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>[MAI211] Probabilités et Statistiques
 (CM)
@@ -4092,16 +4179,16 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -4109,7 +4196,7 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4121,7 +4208,7 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="6" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
@@ -4133,17 +4220,24 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD8
+Prof: Mahfoudh
+Salle: 102</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
 Salle: 202</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -4151,7 +4245,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4163,23 +4257,26 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
 Salle: 201</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Meya
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI1
+Prof: Med Lemine
+Salle: 101 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM Online)
@@ -4187,17 +4284,24 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Meya
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4285,13 +4389,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4303,13 +4407,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4321,13 +4425,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4339,13 +4443,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4357,13 +4461,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4451,13 +4555,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4469,13 +4573,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4487,13 +4591,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4505,13 +4609,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4523,13 +4627,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4617,13 +4721,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4635,13 +4739,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4653,13 +4757,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4671,13 +4775,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4689,13 +4793,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4783,13 +4887,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4801,13 +4905,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4819,13 +4923,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4837,13 +4941,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4855,13 +4959,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4949,13 +5053,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4967,13 +5071,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4985,13 +5089,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5003,13 +5107,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5021,13 +5125,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>

</xml_diff>

<commit_message>
succesfully finished the logic of the classes of type specialite the only thing left is to fix some user interface element
</commit_message>
<xml_diff>
--- a/modele/Tous_les_Emplois_du_Temps.xlsx
+++ b/modele/Tous_les_Emplois_du_Temps.xlsx
@@ -584,26 +584,29 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
 Salle: 101</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
+(TP) - TD1
+Prof: Sidi Mouhamed
+Salle: 102 /// [DEV210] Programmation Python
 (TP) - TD2
 Prof: Esseyssah
-Salle: 102</t>
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -614,14 +617,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
+      <c r="F3" s="7" t="inlineStr"/>
       <c r="G3" s="7" t="inlineStr"/>
       <c r="H3" s="7" t="inlineStr">
         <is>
@@ -646,8 +642,48 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(TP) - TD1
+Prof: Debagh
+Salle: 102 /// [DEV211] Langages Web
+(TP) - TD2
+Prof: Aicha
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>[DPR212] Projet Personnel et Professionnel II
 (CM)
@@ -655,7 +691,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
@@ -663,15 +699,67 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
 Salle: 101</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TD2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (CM)
@@ -679,74 +767,21 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Hassina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI1
+Prof: Med Lemine
+Salle: 101 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 201 /// [RSS210] Services Reseaux
+(TP) - RSS-TD1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TD2
+Prof: Saw
+Salle: 103</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -772,30 +807,7 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(TP) - TD1
-Prof: Debagh
-Salle: 102 /// [DEV211] Langages Web
-(TP) - TD2
-Prof: Aicha
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM) - DSI1
-Prof: Med Lemine
-Salle: 101 /// [CNM210] CMS et PAO
-(CM) - DWM
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (CM)
@@ -803,15 +815,42 @@
 Salle: 101</t>
         </is>
       </c>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI2-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI2-TD2
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
 Salle: 101</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
@@ -2284,9 +2323,26 @@
       </c>
       <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TD2
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM)
+Prof: Med Lemine
+Salle: 101</t>
+        </is>
+      </c>
       <c r="G6" s="7" t="inlineStr"/>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -2301,14 +2357,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM)
-Prof: Med Lemine
-Salle: 101</t>
-        </is>
-      </c>
+      <c r="C7" s="7" t="inlineStr"/>
       <c r="D7" s="7" t="inlineStr"/>
       <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr"/>
@@ -2567,7 +2616,16 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
@@ -2575,32 +2633,20 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
 Salle: 101</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD3
-Prof: Kaber
-Salle: 102 /// [SYR211] Systèmes d’exploitation
-(TP) - TD4
-Prof: Debagh
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Sidi Soueina
-Salle: 201</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr"/>
@@ -2624,22 +2670,172 @@
 Salle: 201 /// [RSS210] Services Reseaux
 (CM) - RSS
 Prof: Souvi
-Salle: 101 /// [DEV210] Programmation Python
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Sidi Soueina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD3
+Prof: Kaber
+Salle: 102 /// [DEV210] Programmation Python
 (TP) - TD4
 Prof: Esseyssah
-Salle: 102</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
 Salle: 201</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TD2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI1
+Prof: Med Lemine
+Salle: 101 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 201 /// [RSS210] Services Reseaux
+(TP) - RSS-TD1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TD2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD3
@@ -2650,155 +2846,34 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
 Salle: 201</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI2-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI2-TD2
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
 Salle: 201</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Hassina
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Debagh
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM) - DSI1
-Prof: Med Lemine
-Salle: 101 /// [CNM210] CMS et PAO
-(CM) - DWM
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr"/>
       <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr">
         <is>
@@ -2953,7 +3028,17 @@
       <c r="C6" s="7" t="inlineStr"/>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(TP) - RSS-TD1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TD2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
       <c r="G6" s="7" t="inlineStr"/>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -3283,9 +3368,23 @@
       </c>
       <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>[CNM210] CMS et PAO
+(TD Online)
+Prof: Cheikhani
+Salle: En ligne</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[CNM210] CMS et PAO
+(CM)
+Prof: Cheikhani
+Salle: 201</t>
+        </is>
+      </c>
       <c r="G6" s="7" t="inlineStr"/>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -3300,14 +3399,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>[CNM210] CMS et PAO
-(CM)
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
+      <c r="C7" s="7" t="inlineStr"/>
       <c r="D7" s="7" t="inlineStr"/>
       <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr"/>
@@ -3482,7 +3574,17 @@
       <c r="B7" s="7" t="inlineStr"/>
       <c r="C7" s="7" t="inlineStr"/>
       <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI2-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI2-TD2
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
       <c r="F7" s="7" t="inlineStr"/>
       <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr">
@@ -3741,10 +3843,10 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 202</t>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 201</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -3752,30 +3854,47 @@
           <t>[DEV211] Langages Web
 (TP) - TD5
 Prof: Meya
-Salle: 102 /// [DEV211] Langages Web
+Salle: 104 /// [DEV211] Langages Web
 (TP) - TD6
 Prof: Aicha
+Salle: 204</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD5
+Prof: Kaber
+Salle: 102 /// [SYR211] Systèmes d’exploitation
+(TP) - TD6
+Prof: Debagh
 Salle: 103</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr"/>
       <c r="E3" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
 Prof: Hatabi
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
 Salle: 201</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 101</t>
+        </is>
+      </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
@@ -3805,10 +3924,41 @@
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Moussa
-Salle: 202</t>
+Salle: 201</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Meya
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>[MAI211] Probabilités et Statistiques
 (CM)
@@ -3816,28 +3966,16 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Meya
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
 Salle: 202</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -3845,25 +3983,6 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
       <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
@@ -3878,62 +3997,43 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
           <t>[DPR211] Anglais II
 (CM)
 Prof: Hatabi
 Salle: 201</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Marba
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TD2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD5
-Prof: Kaber
-Salle: 104 /// [DEV210] Programmation Python
 (TP) - TD6
 Prof: Mahfoudh
-Salle: 204</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
+Salle: 102</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
@@ -3941,34 +4041,72 @@
 Salle: 101 /// [CNM210] CMS et PAO
 (CM) - DWM
 Prof: Cheikhani
+Salle: 201 /// [RSS210] Services Reseaux
+(TP) - RSS-TD1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TD2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
 Salle: 201</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI2-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI2-TD2
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Marba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>[SPEC211] PI 1
 (CM)
 Prof: Encadreur
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
 Salle: 201</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
@@ -4059,53 +4197,53 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
-(TD)
+(CM Online)
 Prof: Marba
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD7
 Prof: Kaber
-Salle: 103 /// [SYR211] Systèmes d’exploitation
+Salle: 102 /// [SYR211] Systèmes d’exploitation
 (TP) - TD8
 Prof: Debagh
-Salle: 104</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
 Salle: 202</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 203</t>
-        </is>
-      </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 101</t>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 201</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -4131,9 +4269,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
@@ -4141,22 +4277,31 @@
 Salle: 202</t>
         </is>
       </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Cheiba
+Salle: 202</t>
+        </is>
+      </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
 Prof: Hatabi
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
-Salle: 203</t>
-        </is>
-      </c>
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr"/>
       <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
@@ -4169,21 +4314,28 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Cheiba
-Salle: 202</t>
-        </is>
-      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD8
+Prof: Mahfoudh
+Salle: 102</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
 Salle: 203</t>
         </is>
       </c>
@@ -4220,52 +4372,29 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TD2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
-(TP) - TD8
-Prof: Mahfoudh
-Salle: 102</t>
+(CM)
+Prof: Moussa
+Salle: 201</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
@@ -4273,32 +4402,70 @@
 Salle: 101 /// [CNM210] CMS et PAO
 (CM) - DWM
 Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
+Salle: 201 /// [RSS210] Services Reseaux
+(TP) - RSS-TD1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TD2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
-(CM Online)
+(TD)
 Prof: Marba
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr">
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI2-TD1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI2-TD2
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>[MAI212] Préparation à la certification PIX 2
 (CM)
 Prof: Meya
 Salle: 202</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 101</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">

</xml_diff>